<commit_message>
feat(saude-fiscal): adiciona notas CAPAG por indicador e filtros de analise
- Modelo IndicadoresAtuais: novos campos capag_indicador_I/II/III_nota,
  rgf_comprometimento_pessoal e rgf_liquidez_relativa (migration 0009)
- Views: filtros capag_campo (nota geral ou indicador I/II/III) e capag_nota,
  com carregamento dinamico dos campos usados no grafico
- Front: novos controles de filtro na home e ajustes no script.js
- Dados: atualiza base CAPAG para capag_12_09_26.xlsx e move as planilhas
  anteriores para base_datas/log/

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/base_datas/crescimento_medio_receita_porte.xlsx
+++ b/base_datas/crescimento_medio_receita_porte.xlsx
@@ -373,7 +373,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>365.170768643801</v>
+        <v>367.1396893692847</v>
       </c>
     </row>
     <row r="3">
@@ -383,7 +383,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>288.6208745049647</v>
+        <v>291.7104963916848</v>
       </c>
     </row>
     <row r="4">
@@ -393,7 +393,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>353.1633725992844</v>
+        <v>353.247477327886</v>
       </c>
     </row>
     <row r="5">
@@ -403,7 +403,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>239.7635833334444</v>
+        <v>239.8010294571989</v>
       </c>
     </row>
     <row r="6">
@@ -413,7 +413,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>339.5332703019551</v>
+        <v>340.2799476275773</v>
       </c>
     </row>
     <row r="7">
@@ -423,7 +423,7 @@
         </is>
       </c>
       <c r="B7">
-        <v>343.2118929331372</v>
+        <v>343.3441336315546</v>
       </c>
     </row>
     <row r="8">
@@ -443,7 +443,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>340.9282456257582</v>
+        <v>341.7298756601739</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: atualiza planilhas de base em 15-09
Regeneracao das bases de populacao, receitas correntes, percentis, medias e
medianas (nacional, UF e porte) e das series de crescimento medio.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/base_datas/crescimento_medio_receita_porte.xlsx
+++ b/base_datas/crescimento_medio_receita_porte.xlsx
@@ -373,7 +373,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>365.170768643801</v>
+        <v>367.1396893692847</v>
       </c>
     </row>
     <row r="3">
@@ -383,7 +383,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>288.6208745049647</v>
+        <v>291.7104963916848</v>
       </c>
     </row>
     <row r="4">
@@ -393,7 +393,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>353.1633725992844</v>
+        <v>353.247477327886</v>
       </c>
     </row>
     <row r="5">
@@ -403,7 +403,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>239.7635833334444</v>
+        <v>239.8010294571989</v>
       </c>
     </row>
     <row r="6">
@@ -413,7 +413,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>339.5332703019551</v>
+        <v>339.9738677530456</v>
       </c>
     </row>
     <row r="7">
@@ -423,7 +423,7 @@
         </is>
       </c>
       <c r="B7">
-        <v>343.2118929331372</v>
+        <v>343.3441336315546</v>
       </c>
     </row>
     <row r="8">
@@ -443,7 +443,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>340.9282456257582</v>
+        <v>341.7298756601739</v>
       </c>
     </row>
   </sheetData>

</xml_diff>